<commit_message>
backup: auto snapshot 2026-06-11 23:49
</commit_message>
<xml_diff>
--- a/SolarOperator_Trust_Distribution_Budget.xlsx
+++ b/SolarOperator_Trust_Distribution_Budget.xlsx
@@ -618,10 +618,11 @@
     <row r="2" ht="26" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Prepared for trustee review · One-time $25,000 distribution · Figures as of June 2026 · STATUS column distinguishes receipt-backed (Documented) costs from forward Estimates.</t>
-        </is>
-      </c>
-    </row>
+          <t>Prepared for trustee review · $25,000 distribution · Figures as of June 2026 · At the current ~$10,000/mo build-phase draw this is ~2.5 months of runway, NOT a one-time top-up. STATUS distinguishes receipt-backed (Documented) costs from forward Estimates.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -632,6 +633,7 @@
         <v>25000</v>
       </c>
     </row>
+    <row r="5"/>
     <row r="6" ht="24" customHeight="1">
       <c r="A6" s="5" t="inlineStr">
         <is>
@@ -675,7 +677,7 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="10" t="inlineStr">
+      <c r="A8" s="28" t="inlineStr">
         <is>
           <t>AI compute — remaining build push</t>
         </is>
@@ -685,17 +687,17 @@
           <t>Forward estimate</t>
         </is>
       </c>
-      <c r="C8" s="12" t="n">
+      <c r="C8" s="29" t="n">
         <v>7000</v>
       </c>
-      <c r="D8" s="13" t="inlineStr">
+      <c r="D8" s="30" t="inlineStr">
         <is>
           <t>Estimate</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="10" t="inlineStr">
+      <c r="A9" s="28" t="inlineStr">
         <is>
           <t>Hosting &amp; infrastructure (≈12 mo)</t>
         </is>
@@ -705,17 +707,17 @@
           <t>Railway, email, auth, data integrations</t>
         </is>
       </c>
-      <c r="C9" s="12" t="n">
+      <c r="C9" s="29" t="n">
         <v>2400</v>
       </c>
-      <c r="D9" s="13" t="inlineStr">
+      <c r="D9" s="30" t="inlineStr">
         <is>
           <t>Estimate</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="10" t="inlineStr">
+      <c r="A10" s="28" t="inlineStr">
         <is>
           <t>Listing &amp; compliance</t>
         </is>
@@ -725,17 +727,17 @@
           <t>Chrome Web Store, registration, misc.</t>
         </is>
       </c>
-      <c r="C10" s="12" t="n">
+      <c r="C10" s="29" t="n">
         <v>750</v>
       </c>
-      <c r="D10" s="13" t="inlineStr">
+      <c r="D10" s="30" t="inlineStr">
         <is>
           <t>Estimate</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="10" t="inlineStr">
+      <c r="A11" s="28" t="inlineStr">
         <is>
           <t>Contingency / buffer to round to ask</t>
         </is>
@@ -745,10 +747,10 @@
           <t>Variance on estimates above</t>
         </is>
       </c>
-      <c r="C11" s="12" t="n">
+      <c r="C11" s="29" t="n">
         <v>3003.3</v>
       </c>
-      <c r="D11" s="13" t="inlineStr">
+      <c r="D11" s="30" t="inlineStr">
         <is>
           <t>Estimate</t>
         </is>
@@ -767,10 +769,11 @@
       </c>
       <c r="D12" s="14" t="n"/>
     </row>
+    <row r="13"/>
     <row r="14">
       <c r="A14" s="16" t="inlineStr">
         <is>
-          <t>Honesty note: $11,846.70 is documented and receipt-backed from the model-provider console. The four Estimate lines are forward projections, not invoices — they are Ford's good-faith planning numbers and may shift. Itemized forward estimates total $10,150.00; the $3,003.30 buffer absorbs estimate variance and rounds the request to the $25,000 figure. Backup detail is on the 'Costs to Date' and 'Use of Funds' tabs.</t>
+          <t>Honesty note: $11,846.70 is documented and receipt-backed from the model-provider console. The product currently draws ~$10,000/mo (compute-dominated) building out utility coverage, so $25,000 is roughly 2.5 months of runway, not a one-time top-up. The four Estimate lines are forward projections, not invoices. Itemized forward estimates total $10,150.00; the $3,003.30 buffer absorbs variance and rounds to $25,000. The draw falls sharply once utility onboarding is done — see 'Path to Self-Sufficiency'.</t>
         </is>
       </c>
     </row>
@@ -913,7 +916,7 @@
           <t>$5.00 standard</t>
         </is>
       </c>
-      <c r="C8" s="12" t="n">
+      <c r="C8" s="29" t="n">
         <v>5</v>
       </c>
       <c r="D8" s="18" t="inlineStr">
@@ -1003,6 +1006,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="24" customHeight="1">
       <c r="A4" s="5" t="inlineStr">
         <is>
@@ -1026,7 +1030,7 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="10" t="inlineStr">
+      <c r="A5" s="28" t="inlineStr">
         <is>
           <t>AI compute — remaining dev push</t>
         </is>
@@ -1036,7 +1040,7 @@
           <t>Agent-swarm work to add utilities for v1 (New England) coverage</t>
         </is>
       </c>
-      <c r="C5" s="12" t="n">
+      <c r="C5" s="29" t="n">
         <v>7000</v>
       </c>
       <c r="D5" s="11" t="inlineStr">
@@ -1046,7 +1050,7 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="10" t="inlineStr">
+      <c r="A6" s="28" t="inlineStr">
         <is>
           <t>Hosting &amp; infrastructure (~12 mo)</t>
         </is>
@@ -1056,7 +1060,7 @@
           <t>Railway containers, email, auth, data integrations</t>
         </is>
       </c>
-      <c r="C6" s="12" t="n">
+      <c r="C6" s="29" t="n">
         <v>2400</v>
       </c>
       <c r="D6" s="11" t="inlineStr">
@@ -1066,7 +1070,7 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="10" t="inlineStr">
+      <c r="A7" s="28" t="inlineStr">
         <is>
           <t>Listing &amp; compliance</t>
         </is>
@@ -1076,7 +1080,7 @@
           <t>Chrome Web Store, business registration, misc. compliance</t>
         </is>
       </c>
-      <c r="C7" s="12" t="n">
+      <c r="C7" s="29" t="n">
         <v>750</v>
       </c>
       <c r="D7" s="11" t="inlineStr">
@@ -1086,7 +1090,7 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="10" t="inlineStr">
+      <c r="A8" s="28" t="inlineStr">
         <is>
           <t>Contingency / buffer</t>
         </is>
@@ -1096,7 +1100,7 @@
           <t>Estimate variance; rounds request to $25,000 ask</t>
         </is>
       </c>
-      <c r="C8" s="12" t="n">
+      <c r="C8" s="29" t="n">
         <v>3003.3</v>
       </c>
       <c r="D8" s="11" t="inlineStr">
@@ -1118,10 +1122,11 @@
       </c>
       <c r="D9" s="20" t="n"/>
     </row>
+    <row r="10"/>
     <row r="11">
       <c r="A11" s="16" t="inlineStr">
         <is>
-          <t>Commitment: this is a one-time disbursement that closes out the build phase. Development-phase compute is front-loaded; once the product settles, ongoing costs drop to a fraction of these figures and live Stripe billing is already in place to cover them.</t>
+          <t>Commitment: this distribution funds the remaining build phase. At the current ~$10,000/mo draw, $25,000 is ~2.5 months of runway. The draw is compute-dominated and one-time per utility — once New England coverage is built it drops to a settled run-rate (~$200/mo + light compute), which live Stripe billing is already wired to cover.</t>
         </is>
       </c>
     </row>
@@ -1166,6 +1171,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="23" t="inlineStr">
         <is>
@@ -1251,6 +1257,7 @@
         </is>
       </c>
     </row>
+    <row r="10"/>
     <row r="11">
       <c r="A11" s="23" t="inlineStr">
         <is>
@@ -1362,10 +1369,11 @@
         </is>
       </c>
     </row>
+    <row r="18"/>
     <row r="19">
       <c r="A19" s="16" t="inlineStr">
         <is>
-          <t>Read this as orders of magnitude, not a forecast. Pricing is live and real; the array counts are scenarios to show the shape of the economics. Quarterly revenue uses the graduated bands. The point: ongoing run-rate after the build phase is modest, and live billing is already wired to cover it — which is why this is a one-time request, not the start of a pattern.</t>
+          <t>Read this as orders of magnitude, not a forecast. Pricing is live and real; array counts are scenarios. IMPORTANT: these counts cover the SETTLED ~$200/mo run-rate, NOT today's ~$10,000/mo build draw. The distribution bridges that gap; the draw must fall as utility onboarding finishes. Live billing is already wired, which is why this is a one-time request, not the start of a pattern.</t>
         </is>
       </c>
     </row>

</xml_diff>